<commit_message>
Update expense breakdown: training /3mo, taxi 1/wk, relationships outings+home
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WQtgSHTUBUwP9xHzFTYxiY
</commit_message>
<xml_diff>
--- a/decomposition_expenses.xlsx
+++ b/decomposition_expenses.xlsx
@@ -537,7 +537,7 @@
     <col width="34" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
     <col width="34" customWidth="1" min="3" max="3"/>
-    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
@@ -674,11 +674,11 @@
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>100 000 ÷ 2,5 мес</t>
+          <t>100 000 ÷ 3 мес</t>
         </is>
       </c>
       <c r="E7" s="6" t="n">
-        <v>40000</v>
+        <v>33333</v>
       </c>
     </row>
     <row r="8">
@@ -773,11 +773,11 @@
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>2/нед × 3 500 туда-обр. ⚠</t>
+          <t>1/нед × 3 500 туда-обр. × 4,33 ⚠</t>
         </is>
       </c>
       <c r="E12" s="6" t="n">
-        <v>30000</v>
+        <v>15000</v>
       </c>
     </row>
     <row r="13">
@@ -1076,16 +1076,16 @@
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>Выходные: кафе, прогулки</t>
+          <t>Выходные: кафе, прогулки, покупки</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>4/мес × 2 000 ⚠</t>
+          <t>4/мес × 6 000 ⚠</t>
         </is>
       </c>
       <c r="E26" s="6" t="n">
-        <v>8000</v>
+        <v>24000</v>
       </c>
     </row>
     <row r="27">
@@ -1098,11 +1098,11 @@
       </c>
       <c r="D27" s="5" t="inlineStr">
         <is>
-          <t>в месяц ⚠</t>
+          <t>в месяц</t>
         </is>
       </c>
       <c r="E27" s="6" t="n">
-        <v>4000</v>
+        <v>30000</v>
       </c>
     </row>
     <row r="28">
@@ -1167,7 +1167,7 @@
     <row r="34">
       <c r="A34" s="11" t="inlineStr">
         <is>
-          <t>Такси и массаж на Бали — прикидка по курсу/тарифам, уточни фактическую стоимость.</t>
+          <t>Отношения: 4 вылазки/мес × 6 000 — если вылазок больше/меньше, поправь.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add per-category explanation column to expense breakdown
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WQtgSHTUBUwP9xHzFTYxiY
</commit_message>
<xml_diff>
--- a/decomposition_expenses.xlsx
+++ b/decomposition_expenses.xlsx
@@ -19,7 +19,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="# ##0 &quot;₽&quot;"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -47,6 +47,10 @@
     <font>
       <b val="1"/>
       <color rgb="00111111"/>
+    </font>
+    <font>
+      <color rgb="00555555"/>
+      <sz val="10"/>
     </font>
     <font>
       <b val="1"/>
@@ -145,7 +149,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -161,11 +165,14 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="7" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="8" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -531,14 +538,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E34"/>
+  <dimension ref="A1:F34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="34" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="32" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="54" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -574,6 +582,11 @@
           <t>₽/мес</t>
         </is>
       </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Пояснение</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
@@ -598,6 +611,11 @@
       <c r="E3" s="6" t="n">
         <v>0</v>
       </c>
+      <c r="F3" s="7" t="inlineStr">
+        <is>
+          <t>Аренда виллы/жилья. Пока не заполнено — обычно самая крупная статья, впиши свою сумму.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -622,6 +640,11 @@
       <c r="E4" s="6" t="n">
         <v>44000</v>
       </c>
+      <c r="F4" s="7" t="inlineStr">
+        <is>
+          <t>Общий долг 266 400 ₽ гасим за 6 месяцев → 44 000/мес. Через полгода строка обнулится.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -646,10 +669,15 @@
       <c r="E5" s="6" t="n">
         <v>5000</v>
       </c>
+      <c r="F5" s="7" t="inlineStr">
+        <is>
+          <t>Регулярное развитие: 2 мастер-класса в месяц (чтобы нащупать направление), танц-движухи раз в месяц и крупное обучение (гипноз/ретрит) 100к раз в 3 месяца = 33 333/мес.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="n"/>
-      <c r="B6" s="7" t="n"/>
+      <c r="A6" s="8" t="n"/>
+      <c r="B6" s="8" t="n"/>
       <c r="C6" s="5" t="inlineStr">
         <is>
           <t>Танцы: рейвы, джемы, съёмки клипа</t>
@@ -663,10 +691,11 @@
       <c r="E6" s="6" t="n">
         <v>2000</v>
       </c>
+      <c r="F6" s="8" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="7" t="n"/>
-      <c r="B7" s="7" t="n"/>
+      <c r="A7" s="8" t="n"/>
+      <c r="B7" s="8" t="n"/>
       <c r="C7" s="5" t="inlineStr">
         <is>
           <t>Обучение (гипноз, ретриты)</t>
@@ -680,6 +709,7 @@
       <c r="E7" s="6" t="n">
         <v>33333</v>
       </c>
+      <c r="F7" s="8" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
@@ -704,10 +734,15 @@
       <c r="E8" s="6" t="n">
         <v>5000</v>
       </c>
+      <c r="F8" s="7" t="inlineStr">
+        <is>
+          <t>Массаж 2 раза в месяц, курс бадов (15к на 3 мес = 5к/мес), микродозинг и прочие процедуры.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
-      <c r="A9" s="7" t="n"/>
-      <c r="B9" s="7" t="n"/>
+      <c r="A9" s="8" t="n"/>
+      <c r="B9" s="8" t="n"/>
       <c r="C9" s="5" t="inlineStr">
         <is>
           <t>Бады</t>
@@ -721,10 +756,11 @@
       <c r="E9" s="6" t="n">
         <v>5000</v>
       </c>
+      <c r="F9" s="8" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="7" t="n"/>
-      <c r="B10" s="7" t="n"/>
+      <c r="A10" s="8" t="n"/>
+      <c r="B10" s="8" t="n"/>
       <c r="C10" s="5" t="inlineStr">
         <is>
           <t>Мухоморы и прочее</t>
@@ -738,6 +774,7 @@
       <c r="E10" s="6" t="n">
         <v>3000</v>
       </c>
+      <c r="F10" s="8" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
@@ -762,10 +799,15 @@
       <c r="E11" s="6" t="n">
         <v>10000</v>
       </c>
+      <c r="F11" s="7" t="inlineStr">
+        <is>
+          <t>Аренда байка помесячно + такси до Nuanu раз в неделю (туда-обратно ≈ 3 500, ×4,33 недели).</t>
+        </is>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" s="7" t="n"/>
-      <c r="B12" s="7" t="n"/>
+      <c r="A12" s="8" t="n"/>
+      <c r="B12" s="8" t="n"/>
       <c r="C12" s="5" t="inlineStr">
         <is>
           <t>Такси Nusa Dua ↔ Nuanu</t>
@@ -779,6 +821,7 @@
       <c r="E12" s="6" t="n">
         <v>15000</v>
       </c>
+      <c r="F12" s="8" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
@@ -803,6 +846,11 @@
       <c r="E13" s="6" t="n">
         <v>10000</v>
       </c>
+      <c r="F13" s="7" t="inlineStr">
+        <is>
+          <t>Качественная одежда и уход за собой, ~10к в месяц.</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
@@ -827,10 +875,15 @@
       <c r="E14" s="6" t="n">
         <v>10000</v>
       </c>
+      <c r="F14" s="7" t="inlineStr">
+        <is>
+          <t>Разовая закупка (монитор 2K, колонки, 16 ГБ RAM ≈ 30к) растянута на 3 мес + оператор связи/интернет. После закупки строка снизится до ~2к.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
-      <c r="A15" s="7" t="n"/>
-      <c r="B15" s="7" t="n"/>
+      <c r="A15" s="8" t="n"/>
+      <c r="B15" s="8" t="n"/>
       <c r="C15" s="5" t="inlineStr">
         <is>
           <t>Связь + домашний интернет</t>
@@ -844,6 +897,7 @@
       <c r="E15" s="6" t="n">
         <v>2000</v>
       </c>
+      <c r="F15" s="8" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
@@ -868,6 +922,11 @@
       <c r="E16" s="6" t="n">
         <v>0</v>
       </c>
+      <c r="F16" s="7" t="inlineStr">
+        <is>
+          <t>Траты на личный бренд: реклама, съёмки, монтаж, подрядчики. Пока не заполнено — впиши, если есть.</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
@@ -892,10 +951,15 @@
       <c r="E17" s="6" t="n">
         <v>16000</v>
       </c>
+      <c r="F17" s="7" t="inlineStr">
+        <is>
+          <t>8 выходов в рестораны/кафе (~2к чек) + продукты домой + доставка.</t>
+        </is>
+      </c>
     </row>
     <row r="18">
-      <c r="A18" s="7" t="n"/>
-      <c r="B18" s="7" t="n"/>
+      <c r="A18" s="8" t="n"/>
+      <c r="B18" s="8" t="n"/>
       <c r="C18" s="5" t="inlineStr">
         <is>
           <t>Продукты</t>
@@ -909,10 +973,11 @@
       <c r="E18" s="6" t="n">
         <v>12000</v>
       </c>
+      <c r="F18" s="8" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="7" t="n"/>
-      <c r="B19" s="7" t="n"/>
+      <c r="A19" s="8" t="n"/>
+      <c r="B19" s="8" t="n"/>
       <c r="C19" s="5" t="inlineStr">
         <is>
           <t>Доставка</t>
@@ -926,6 +991,7 @@
       <c r="E19" s="6" t="n">
         <v>2000</v>
       </c>
+      <c r="F19" s="8" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
@@ -950,10 +1016,15 @@
       <c r="E20" s="6" t="n">
         <v>5000</v>
       </c>
+      <c r="F20" s="7" t="inlineStr">
+        <is>
+          <t>Подарки родным и девушке, по 5к на каждого = 10к/мес.</t>
+        </is>
+      </c>
     </row>
     <row r="21">
-      <c r="A21" s="7" t="n"/>
-      <c r="B21" s="7" t="n"/>
+      <c r="A21" s="8" t="n"/>
+      <c r="B21" s="8" t="n"/>
       <c r="C21" s="5" t="inlineStr">
         <is>
           <t>Девушке</t>
@@ -967,6 +1038,7 @@
       <c r="E21" s="6" t="n">
         <v>5000</v>
       </c>
+      <c r="F21" s="8" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
@@ -991,6 +1063,11 @@
       <c r="E22" s="6" t="n">
         <v>33333</v>
       </c>
+      <c r="F22" s="7" t="inlineStr">
+        <is>
+          <t>Крупный отдых/отпуск 100к раз в 3 месяца → 33 333/мес.</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
@@ -1015,6 +1092,11 @@
       <c r="E23" s="6" t="n">
         <v>3000</v>
       </c>
+      <c r="F23" s="7" t="inlineStr">
+        <is>
+          <t>Приложения, музыка, кино и прочие подписки, ~3к/мес.</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
@@ -1039,6 +1121,11 @@
       <c r="E24" s="6" t="n">
         <v>20000</v>
       </c>
+      <c r="F24" s="7" t="inlineStr">
+        <is>
+          <t>Продление/визаран на Бали. Цифра перенесена из прошлой версии — подтверди.</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
@@ -1063,6 +1150,11 @@
       <c r="E25" s="6" t="n">
         <v>5000</v>
       </c>
+      <c r="F25" s="7" t="inlineStr">
+        <is>
+          <t>Регулярные пожертвования, 5к/мес.</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
@@ -1087,10 +1179,15 @@
       <c r="E26" s="6" t="n">
         <v>24000</v>
       </c>
+      <c r="F26" s="7" t="inlineStr">
+        <is>
+          <t>Совместные вылазки по выходным (мин. 5–6к за раз, ~4 раза/мес) + совместный быт дома 30к. Проверь: если быт включает продукты — часть пересекается с «Питанием».</t>
+        </is>
+      </c>
     </row>
     <row r="27">
-      <c r="A27" s="7" t="n"/>
-      <c r="B27" s="7" t="n"/>
+      <c r="A27" s="8" t="n"/>
+      <c r="B27" s="8" t="n"/>
       <c r="C27" s="5" t="inlineStr">
         <is>
           <t>Совместный быт дома</t>
@@ -1104,6 +1201,7 @@
       <c r="E27" s="6" t="n">
         <v>30000</v>
       </c>
+      <c r="F27" s="8" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
@@ -1128,69 +1226,82 @@
       <c r="E28" s="6" t="n">
         <v>0</v>
       </c>
+      <c r="F28" s="7" t="inlineStr">
+        <is>
+          <t>Пока не заполнено. Уточни, чем отличается от «Отдыха» — если это перелёты (Азия/домой), посчитаем отдельно.</t>
+        </is>
+      </c>
     </row>
     <row r="29">
-      <c r="A29" s="8" t="inlineStr">
+      <c r="A29" s="9" t="inlineStr">
         <is>
           <t>ИТОГО расходов / мес</t>
         </is>
       </c>
-      <c r="B29" s="9">
+      <c r="B29" s="10">
         <f>SUM(E3:E28)</f>
         <v/>
       </c>
-      <c r="C29" s="10" t="n"/>
-      <c r="D29" s="10" t="n"/>
-      <c r="E29" s="10" t="n"/>
+      <c r="C29" s="11" t="n"/>
+      <c r="D29" s="11" t="n"/>
+      <c r="E29" s="11" t="n"/>
+      <c r="F29" s="11" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="11" t="inlineStr">
+      <c r="A31" s="12" t="inlineStr">
         <is>
           <t>⚠ — оценка/допущение, поправь под себя. Разовые покупки делятся на срок (÷ мес).</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="11" t="inlineStr">
+      <c r="A32" s="12" t="inlineStr">
         <is>
           <t>Не заполнено (нужны твои цифры): Жильё, Бизнес (личный бренд), Поездки.</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="11" t="inlineStr">
+      <c r="A33" s="12" t="inlineStr">
         <is>
           <t>«Отдых» и «Поездки» пока дублируют смысл — уточни разницу, иначе объединим.</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="11" t="inlineStr">
+      <c r="A34" s="12" t="inlineStr">
         <is>
           <t>Отношения: 4 вылазки/мес × 6 000 — если вылазок больше/меньше, поправь.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="20">
-    <mergeCell ref="A34:E34"/>
+  <mergeCells count="27">
+    <mergeCell ref="F17:F19"/>
     <mergeCell ref="A8:A10"/>
     <mergeCell ref="A17:A19"/>
     <mergeCell ref="A29"/>
     <mergeCell ref="B11:B12"/>
-    <mergeCell ref="A1:E1"/>
     <mergeCell ref="A5:A7"/>
+    <mergeCell ref="F20:F21"/>
     <mergeCell ref="B14:B15"/>
     <mergeCell ref="B5:B7"/>
+    <mergeCell ref="F8:F10"/>
+    <mergeCell ref="A33:F33"/>
+    <mergeCell ref="F26:F27"/>
     <mergeCell ref="A26:A27"/>
+    <mergeCell ref="A32:F32"/>
     <mergeCell ref="A14:A15"/>
-    <mergeCell ref="A33:E33"/>
+    <mergeCell ref="A31:F31"/>
     <mergeCell ref="A20:A21"/>
+    <mergeCell ref="A34:F34"/>
     <mergeCell ref="B8:B10"/>
     <mergeCell ref="B20:B21"/>
-    <mergeCell ref="A32:E32"/>
+    <mergeCell ref="F5:F7"/>
+    <mergeCell ref="F11:F12"/>
+    <mergeCell ref="F14:F15"/>
     <mergeCell ref="B17:B19"/>
-    <mergeCell ref="A31:E31"/>
+    <mergeCell ref="A1:F1"/>
     <mergeCell ref="B26:B27"/>
     <mergeCell ref="A11:A12"/>
   </mergeCells>

</xml_diff>

<commit_message>
Add per-item detailed cost math; split gadgets into devices
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WQtgSHTUBUwP9xHzFTYxiY
</commit_message>
<xml_diff>
--- a/decomposition_expenses.xlsx
+++ b/decomposition_expenses.xlsx
@@ -149,7 +149,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -164,6 +164,9 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -538,15 +541,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F34"/>
+  <dimension ref="A1:F35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
-    <col width="32" customWidth="1" min="3" max="3"/>
-    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="46" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="54" customWidth="1" min="6" max="6"/>
+    <col width="50" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -569,12 +572,12 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Детализация</t>
+          <t>Пункт</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Расчёт / период</t>
+          <t>Подробный расчёт стоимости</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -603,17 +606,17 @@
           <t>Аренда жилья</t>
         </is>
       </c>
-      <c r="D3" s="5" t="inlineStr">
-        <is>
-          <t>⚠ уточни сумму</t>
-        </is>
-      </c>
-      <c r="E3" s="6" t="n">
+      <c r="D3" s="6" t="inlineStr">
+        <is>
+          <t>⚠ уточни сумму аренды в месяц</t>
+        </is>
+      </c>
+      <c r="E3" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="F3" s="7" t="inlineStr">
-        <is>
-          <t>Аренда виллы/жилья. Пока не заполнено — обычно самая крупная статья, впиши свою сумму.</t>
+      <c r="F3" s="8" t="inlineStr">
+        <is>
+          <t>Аренда виллы/жилья. Пока не заполнено — обычно самая крупная статья.</t>
         </is>
       </c>
     </row>
@@ -632,17 +635,17 @@
           <t>Погашение долга</t>
         </is>
       </c>
-      <c r="D4" s="5" t="inlineStr">
-        <is>
-          <t>266 400 ÷ 6 мес</t>
-        </is>
-      </c>
-      <c r="E4" s="6" t="n">
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>266 400 ₽ (весь долг) ÷ 6 мес = 44 000 ₽/мес</t>
+        </is>
+      </c>
+      <c r="E4" s="7" t="n">
         <v>44000</v>
       </c>
-      <c r="F4" s="7" t="inlineStr">
-        <is>
-          <t>Общий долг 266 400 ₽ гасим за 6 месяцев → 44 000/мес. Через полгода строка обнулится.</t>
+      <c r="F4" s="8" t="inlineStr">
+        <is>
+          <t>Гасим весь долг 266 400 ₽ за 6 месяцев. Через полгода строка обнулится.</t>
         </is>
       </c>
     </row>
@@ -661,55 +664,55 @@
           <t>Мастер-классы</t>
         </is>
       </c>
-      <c r="D5" s="5" t="inlineStr">
-        <is>
-          <t>2/мес × 2 500 ⚠</t>
-        </is>
-      </c>
-      <c r="E5" s="6" t="n">
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>2 шт/мес × 2 500 ₽ = 5 000 ₽ ⚠</t>
+        </is>
+      </c>
+      <c r="E5" s="7" t="n">
         <v>5000</v>
       </c>
-      <c r="F5" s="7" t="inlineStr">
-        <is>
-          <t>Регулярное развитие: 2 мастер-класса в месяц (чтобы нащупать направление), танц-движухи раз в месяц и крупное обучение (гипноз/ретрит) 100к раз в 3 месяца = 33 333/мес.</t>
+      <c r="F5" s="8" t="inlineStr">
+        <is>
+          <t>Регулярное развитие: мастер-классы, танц-движухи и крупное обучение раз в 3 месяца.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="8" t="n"/>
-      <c r="B6" s="8" t="n"/>
+      <c r="A6" s="9" t="n"/>
+      <c r="B6" s="9" t="n"/>
       <c r="C6" s="5" t="inlineStr">
         <is>
           <t>Танцы: рейвы, джемы, съёмки клипа</t>
         </is>
       </c>
-      <c r="D6" s="5" t="inlineStr">
-        <is>
-          <t>1/мес × 2 000 ⚠</t>
-        </is>
-      </c>
-      <c r="E6" s="6" t="n">
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>1 событие/мес × 2 000 ₽ = 2 000 ₽ ⚠</t>
+        </is>
+      </c>
+      <c r="E6" s="7" t="n">
         <v>2000</v>
       </c>
-      <c r="F6" s="8" t="n"/>
+      <c r="F6" s="9" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="8" t="n"/>
-      <c r="B7" s="8" t="n"/>
+      <c r="A7" s="9" t="n"/>
+      <c r="B7" s="9" t="n"/>
       <c r="C7" s="5" t="inlineStr">
         <is>
           <t>Обучение (гипноз, ретриты)</t>
         </is>
       </c>
-      <c r="D7" s="5" t="inlineStr">
-        <is>
-          <t>100 000 ÷ 3 мес</t>
-        </is>
-      </c>
-      <c r="E7" s="6" t="n">
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>100 000 ₽ раз в 3 мес ÷ 3 = 33 333 ₽/мес</t>
+        </is>
+      </c>
+      <c r="E7" s="7" t="n">
         <v>33333</v>
       </c>
-      <c r="F7" s="8" t="n"/>
+      <c r="F7" s="9" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
@@ -726,55 +729,55 @@
           <t>Массаж</t>
         </is>
       </c>
-      <c r="D8" s="5" t="inlineStr">
-        <is>
-          <t>2/мес × 2 500 ⚠</t>
-        </is>
-      </c>
-      <c r="E8" s="6" t="n">
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>2 раза/мес × 2 500 ₽ = 5 000 ₽ ⚠</t>
+        </is>
+      </c>
+      <c r="E8" s="7" t="n">
         <v>5000</v>
       </c>
-      <c r="F8" s="7" t="inlineStr">
-        <is>
-          <t>Массаж 2 раза в месяц, курс бадов (15к на 3 мес = 5к/мес), микродозинг и прочие процедуры.</t>
+      <c r="F8" s="8" t="inlineStr">
+        <is>
+          <t>Массаж 2 раза в месяц, курс бадов на 3 месяца, микродозинг и процедуры.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="8" t="n"/>
-      <c r="B9" s="8" t="n"/>
+      <c r="A9" s="9" t="n"/>
+      <c r="B9" s="9" t="n"/>
       <c r="C9" s="5" t="inlineStr">
         <is>
           <t>Бады</t>
         </is>
       </c>
-      <c r="D9" s="5" t="inlineStr">
-        <is>
-          <t>15 000 ÷ 3 мес</t>
-        </is>
-      </c>
-      <c r="E9" s="6" t="n">
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>15 000 ₽ (курс на 3 мес) ÷ 3 = 5 000 ₽/мес</t>
+        </is>
+      </c>
+      <c r="E9" s="7" t="n">
         <v>5000</v>
       </c>
-      <c r="F9" s="8" t="n"/>
+      <c r="F9" s="9" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="8" t="n"/>
-      <c r="B10" s="8" t="n"/>
+      <c r="A10" s="9" t="n"/>
+      <c r="B10" s="9" t="n"/>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>Мухоморы и прочее</t>
-        </is>
-      </c>
-      <c r="D10" s="5" t="inlineStr">
-        <is>
-          <t>≈ ⚠</t>
-        </is>
-      </c>
-      <c r="E10" s="6" t="n">
+          <t>Мухоморы, микродозинг и прочее</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="inlineStr">
+        <is>
+          <t>≈ 3 000 ₽/мес ⚠</t>
+        </is>
+      </c>
+      <c r="E10" s="7" t="n">
         <v>3000</v>
       </c>
-      <c r="F10" s="8" t="n"/>
+      <c r="F10" s="9" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
@@ -791,37 +794,37 @@
           <t>Аренда байка</t>
         </is>
       </c>
-      <c r="D11" s="5" t="inlineStr">
-        <is>
-          <t>в месяц ⚠</t>
-        </is>
-      </c>
-      <c r="E11" s="6" t="n">
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>≈ 10 000 ₽/мес ⚠</t>
+        </is>
+      </c>
+      <c r="E11" s="7" t="n">
         <v>10000</v>
       </c>
-      <c r="F11" s="7" t="inlineStr">
-        <is>
-          <t>Аренда байка помесячно + такси до Nuanu раз в неделю (туда-обратно ≈ 3 500, ×4,33 недели).</t>
+      <c r="F11" s="8" t="inlineStr">
+        <is>
+          <t>Аренда байка помесячно + такси до Nuanu раз в неделю (туда-обратно).</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="8" t="n"/>
-      <c r="B12" s="8" t="n"/>
+      <c r="A12" s="9" t="n"/>
+      <c r="B12" s="9" t="n"/>
       <c r="C12" s="5" t="inlineStr">
         <is>
           <t>Такси Nusa Dua ↔ Nuanu</t>
         </is>
       </c>
-      <c r="D12" s="5" t="inlineStr">
-        <is>
-          <t>1/нед × 3 500 туда-обр. × 4,33 ⚠</t>
-        </is>
-      </c>
-      <c r="E12" s="6" t="n">
+      <c r="D12" s="6" t="inlineStr">
+        <is>
+          <t>1 750 ₽ × 2 = 3 500 ₽ туда-обр. × 4,33 нед = 15 000 ₽ ⚠</t>
+        </is>
+      </c>
+      <c r="E12" s="7" t="n">
         <v>15000</v>
       </c>
-      <c r="F12" s="8" t="n"/>
+      <c r="F12" s="9" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
@@ -835,20 +838,20 @@
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>Качественная одежда</t>
-        </is>
-      </c>
-      <c r="D13" s="5" t="inlineStr">
-        <is>
-          <t>в месяц</t>
-        </is>
-      </c>
-      <c r="E13" s="6" t="n">
+          <t>Качественная одежда и уход</t>
+        </is>
+      </c>
+      <c r="D13" s="6" t="inlineStr">
+        <is>
+          <t>≈ 10 000 ₽/мес</t>
+        </is>
+      </c>
+      <c r="E13" s="7" t="n">
         <v>10000</v>
       </c>
-      <c r="F13" s="7" t="inlineStr">
-        <is>
-          <t>Качественная одежда и уход за собой, ~10к в месяц.</t>
+      <c r="F13" s="8" t="inlineStr">
+        <is>
+          <t>Качественная одежда и уход за собой.</t>
         </is>
       </c>
     </row>
@@ -859,249 +862,227 @@
         </is>
       </c>
       <c r="B14" s="4">
-        <f>SUM(E14:E15)</f>
+        <f>SUM(E14:E17)</f>
         <v/>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>Монитор 2K + колонки + 16 ГБ RAM</t>
-        </is>
-      </c>
-      <c r="D14" s="5" t="inlineStr">
-        <is>
-          <t>≈30 000 ÷ 3 мес ⚠</t>
-        </is>
-      </c>
-      <c r="E14" s="6" t="n">
-        <v>10000</v>
-      </c>
-      <c r="F14" s="7" t="inlineStr">
-        <is>
-          <t>Разовая закупка (монитор 2K, колонки, 16 ГБ RAM ≈ 30к) растянута на 3 мес + оператор связи/интернет. После закупки строка снизится до ~2к.</t>
+          <t>Монитор 2K</t>
+        </is>
+      </c>
+      <c r="D14" s="6" t="inlineStr">
+        <is>
+          <t>≈ 20 000 ₽ разово ÷ 3 мес = 6 667 ₽/мес ⚠</t>
+        </is>
+      </c>
+      <c r="E14" s="7" t="n">
+        <v>6667</v>
+      </c>
+      <c r="F14" s="8" t="inlineStr">
+        <is>
+          <t>Разовая закупка железа (≈30 000 ₽) растянута на 3 мес + связь/интернет. После закупки строка упадёт до ~2 000 ₽.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="8" t="n"/>
-      <c r="B15" s="8" t="n"/>
+      <c r="A15" s="9" t="n"/>
+      <c r="B15" s="9" t="n"/>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>Связь + домашний интернет</t>
-        </is>
-      </c>
-      <c r="D15" s="5" t="inlineStr">
-        <is>
-          <t>в месяц ⚠</t>
-        </is>
-      </c>
-      <c r="E15" s="6" t="n">
+          <t>Колонки</t>
+        </is>
+      </c>
+      <c r="D15" s="6" t="inlineStr">
+        <is>
+          <t>≈ 5 000 ₽ разово ÷ 3 мес = 1 667 ₽/мес ⚠</t>
+        </is>
+      </c>
+      <c r="E15" s="7" t="n">
+        <v>1667</v>
+      </c>
+      <c r="F15" s="9" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="9" t="n"/>
+      <c r="B16" s="9" t="n"/>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>Оперативка 16 ГБ</t>
+        </is>
+      </c>
+      <c r="D16" s="6" t="inlineStr">
+        <is>
+          <t>≈ 5 000 ₽ разово ÷ 3 мес = 1 666 ₽/мес ⚠</t>
+        </is>
+      </c>
+      <c r="E16" s="7" t="n">
+        <v>1666</v>
+      </c>
+      <c r="F16" s="9" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="9" t="n"/>
+      <c r="B17" s="9" t="n"/>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>Оператор связи + домашний интернет</t>
+        </is>
+      </c>
+      <c r="D17" s="6" t="inlineStr">
+        <is>
+          <t>≈ 2 000 ₽/мес ⚠</t>
+        </is>
+      </c>
+      <c r="E17" s="7" t="n">
         <v>2000</v>
       </c>
-      <c r="F15" s="8" t="n"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="3" t="inlineStr">
+      <c r="F17" s="9" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
         <is>
           <t>Бизнес (личный бренд)</t>
         </is>
       </c>
-      <c r="B16" s="4">
-        <f>SUM(E16:E16)</f>
-        <v/>
-      </c>
-      <c r="C16" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D16" s="5" t="inlineStr">
+      <c r="B18" s="4">
+        <f>SUM(E18:E18)</f>
+        <v/>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>Реклама, съёмки, подрядчики</t>
+        </is>
+      </c>
+      <c r="D18" s="6" t="inlineStr">
         <is>
           <t>⚠ уточни</t>
         </is>
       </c>
-      <c r="E16" s="6" t="n">
+      <c r="E18" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="F16" s="7" t="inlineStr">
-        <is>
-          <t>Траты на личный бренд: реклама, съёмки, монтаж, подрядчики. Пока не заполнено — впиши, если есть.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="3" t="inlineStr">
+      <c r="F18" s="8" t="inlineStr">
+        <is>
+          <t>Траты на личный бренд: реклама, съёмки, монтаж, подрядчики. Пока не заполнено.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
         <is>
           <t>Питание</t>
         </is>
       </c>
-      <c r="B17" s="4">
-        <f>SUM(E17:E19)</f>
-        <v/>
-      </c>
-      <c r="C17" s="5" t="inlineStr">
+      <c r="B19" s="4">
+        <f>SUM(E19:E21)</f>
+        <v/>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
         <is>
           <t>Рестораны / кафе</t>
         </is>
       </c>
-      <c r="D17" s="5" t="inlineStr">
-        <is>
-          <t>8/мес × 2 000 ⚠</t>
-        </is>
-      </c>
-      <c r="E17" s="6" t="n">
+      <c r="D19" s="6" t="inlineStr">
+        <is>
+          <t>8 раз/мес × 2 000 ₽ = 16 000 ₽ ⚠</t>
+        </is>
+      </c>
+      <c r="E19" s="7" t="n">
         <v>16000</v>
       </c>
-      <c r="F17" s="7" t="inlineStr">
-        <is>
-          <t>8 выходов в рестораны/кафе (~2к чек) + продукты домой + доставка.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="8" t="n"/>
-      <c r="B18" s="8" t="n"/>
-      <c r="C18" s="5" t="inlineStr">
+      <c r="F19" s="8" t="inlineStr">
+        <is>
+          <t>8 выходов в рестораны/кафе + продукты домой + доставка.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="9" t="n"/>
+      <c r="B20" s="9" t="n"/>
+      <c r="C20" s="5" t="inlineStr">
         <is>
           <t>Продукты</t>
         </is>
       </c>
-      <c r="D18" s="5" t="inlineStr">
-        <is>
-          <t>в месяц ⚠</t>
-        </is>
-      </c>
-      <c r="E18" s="6" t="n">
+      <c r="D20" s="6" t="inlineStr">
+        <is>
+          <t>≈ 12 000 ₽/мес ⚠</t>
+        </is>
+      </c>
+      <c r="E20" s="7" t="n">
         <v>12000</v>
       </c>
-      <c r="F18" s="8" t="n"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="8" t="n"/>
-      <c r="B19" s="8" t="n"/>
-      <c r="C19" s="5" t="inlineStr">
+      <c r="F20" s="9" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="9" t="n"/>
+      <c r="B21" s="9" t="n"/>
+      <c r="C21" s="5" t="inlineStr">
         <is>
           <t>Доставка</t>
         </is>
       </c>
-      <c r="D19" s="5" t="inlineStr">
-        <is>
-          <t>в месяц ⚠</t>
-        </is>
-      </c>
-      <c r="E19" s="6" t="n">
+      <c r="D21" s="6" t="inlineStr">
+        <is>
+          <t>≈ 2 000 ₽/мес ⚠</t>
+        </is>
+      </c>
+      <c r="E21" s="7" t="n">
         <v>2000</v>
       </c>
-      <c r="F19" s="8" t="n"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="3" t="inlineStr">
-        <is>
-          <t>Подарки (родным, девушке)</t>
-        </is>
-      </c>
-      <c r="B20" s="4">
-        <f>SUM(E20:E21)</f>
-        <v/>
-      </c>
-      <c r="C20" s="5" t="inlineStr">
-        <is>
-          <t>Родным</t>
-        </is>
-      </c>
-      <c r="D20" s="5" t="inlineStr">
-        <is>
-          <t>в месяц</t>
-        </is>
-      </c>
-      <c r="E20" s="6" t="n">
-        <v>5000</v>
-      </c>
-      <c r="F20" s="7" t="inlineStr">
-        <is>
-          <t>Подарки родным и девушке, по 5к на каждого = 10к/мес.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="8" t="n"/>
-      <c r="B21" s="8" t="n"/>
-      <c r="C21" s="5" t="inlineStr">
-        <is>
-          <t>Девушке</t>
-        </is>
-      </c>
-      <c r="D21" s="5" t="inlineStr">
-        <is>
-          <t>в месяц</t>
-        </is>
-      </c>
-      <c r="E21" s="6" t="n">
-        <v>5000</v>
-      </c>
-      <c r="F21" s="8" t="n"/>
+      <c r="F21" s="9" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>Отдых (выходные, отпуск)</t>
+          <t>Подарки (родным, девушке)</t>
         </is>
       </c>
       <c r="B22" s="4">
-        <f>SUM(E22:E22)</f>
+        <f>SUM(E22:E23)</f>
         <v/>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>Отпуск / вылазки</t>
-        </is>
-      </c>
-      <c r="D22" s="5" t="inlineStr">
-        <is>
-          <t>100 000 ÷ 3 мес</t>
-        </is>
-      </c>
-      <c r="E22" s="6" t="n">
-        <v>33333</v>
-      </c>
-      <c r="F22" s="7" t="inlineStr">
-        <is>
-          <t>Крупный отдых/отпуск 100к раз в 3 месяца → 33 333/мес.</t>
+          <t>Родным</t>
+        </is>
+      </c>
+      <c r="D22" s="6" t="inlineStr">
+        <is>
+          <t>≈ 5 000 ₽/мес</t>
+        </is>
+      </c>
+      <c r="E22" s="7" t="n">
+        <v>5000</v>
+      </c>
+      <c r="F22" s="8" t="inlineStr">
+        <is>
+          <t>Подарки родным и девушке, по 5 000 ₽ = 10 000 ₽/мес.</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="3" t="inlineStr">
-        <is>
-          <t>Подписки услуг</t>
-        </is>
-      </c>
-      <c r="B23" s="4">
-        <f>SUM(E23:E23)</f>
-        <v/>
-      </c>
+      <c r="A23" s="9" t="n"/>
+      <c r="B23" s="9" t="n"/>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>Приложения, музыка, кино</t>
-        </is>
-      </c>
-      <c r="D23" s="5" t="inlineStr">
-        <is>
-          <t>в месяц</t>
-        </is>
-      </c>
-      <c r="E23" s="6" t="n">
-        <v>3000</v>
-      </c>
-      <c r="F23" s="7" t="inlineStr">
-        <is>
-          <t>Приложения, музыка, кино и прочие подписки, ~3к/мес.</t>
-        </is>
-      </c>
+          <t>Девушке</t>
+        </is>
+      </c>
+      <c r="D23" s="6" t="inlineStr">
+        <is>
+          <t>≈ 5 000 ₽/мес</t>
+        </is>
+      </c>
+      <c r="E23" s="7" t="n">
+        <v>5000</v>
+      </c>
+      <c r="F23" s="9" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>Визы (визараны)</t>
+          <t>Отдых (выходные, отпуск)</t>
         </is>
       </c>
       <c r="B24" s="4">
@@ -1110,27 +1091,27 @@
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>Визаран / продление</t>
-        </is>
-      </c>
-      <c r="D24" s="5" t="inlineStr">
-        <is>
-          <t>из прошлой версии ⚠</t>
-        </is>
-      </c>
-      <c r="E24" s="6" t="n">
-        <v>20000</v>
-      </c>
-      <c r="F24" s="7" t="inlineStr">
-        <is>
-          <t>Продление/визаран на Бали. Цифра перенесена из прошлой версии — подтверди.</t>
+          <t>Отпуск / крупная вылазка</t>
+        </is>
+      </c>
+      <c r="D24" s="6" t="inlineStr">
+        <is>
+          <t>100 000 ₽ раз в 3 мес ÷ 3 = 33 333 ₽/мес</t>
+        </is>
+      </c>
+      <c r="E24" s="7" t="n">
+        <v>33333</v>
+      </c>
+      <c r="F24" s="8" t="inlineStr">
+        <is>
+          <t>Крупный отдых/отпуск 100 000 ₽ раз в 3 месяца.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>Благотворительность</t>
+          <t>Подписки услуг</t>
         </is>
       </c>
       <c r="B25" s="4">
@@ -1139,170 +1120,220 @@
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>Пожертвования</t>
-        </is>
-      </c>
-      <c r="D25" s="5" t="inlineStr">
-        <is>
-          <t>в месяц</t>
-        </is>
-      </c>
-      <c r="E25" s="6" t="n">
-        <v>5000</v>
-      </c>
-      <c r="F25" s="7" t="inlineStr">
-        <is>
-          <t>Регулярные пожертвования, 5к/мес.</t>
+          <t>Приложения, музыка, кино</t>
+        </is>
+      </c>
+      <c r="D25" s="6" t="inlineStr">
+        <is>
+          <t>≈ 3 000 ₽/мес</t>
+        </is>
+      </c>
+      <c r="E25" s="7" t="n">
+        <v>3000</v>
+      </c>
+      <c r="F25" s="8" t="inlineStr">
+        <is>
+          <t>Приложения, музыка, кино и прочие подписки.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t>Отношения (быт, совместное время)</t>
+          <t>Визы (визараны)</t>
         </is>
       </c>
       <c r="B26" s="4">
-        <f>SUM(E26:E27)</f>
+        <f>SUM(E26:E26)</f>
         <v/>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>Выходные: кафе, прогулки, покупки</t>
-        </is>
-      </c>
-      <c r="D26" s="5" t="inlineStr">
-        <is>
-          <t>4/мес × 6 000 ⚠</t>
-        </is>
-      </c>
-      <c r="E26" s="6" t="n">
-        <v>24000</v>
-      </c>
-      <c r="F26" s="7" t="inlineStr">
-        <is>
-          <t>Совместные вылазки по выходным (мин. 5–6к за раз, ~4 раза/мес) + совместный быт дома 30к. Проверь: если быт включает продукты — часть пересекается с «Питанием».</t>
+          <t>Визаран / продление визы</t>
+        </is>
+      </c>
+      <c r="D26" s="6" t="inlineStr">
+        <is>
+          <t>≈ 20 000 ₽/мес ⚠ (перенос, подтверди)</t>
+        </is>
+      </c>
+      <c r="E26" s="7" t="n">
+        <v>20000</v>
+      </c>
+      <c r="F26" s="8" t="inlineStr">
+        <is>
+          <t>Продление/визаран на Бали. Цифра перенесена — подтверди.</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="8" t="n"/>
-      <c r="B27" s="8" t="n"/>
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>Благотворительность</t>
+        </is>
+      </c>
+      <c r="B27" s="4">
+        <f>SUM(E27:E27)</f>
+        <v/>
+      </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>Совместный быт дома</t>
-        </is>
-      </c>
-      <c r="D27" s="5" t="inlineStr">
-        <is>
-          <t>в месяц</t>
-        </is>
-      </c>
-      <c r="E27" s="6" t="n">
-        <v>30000</v>
-      </c>
-      <c r="F27" s="8" t="n"/>
+          <t>Пожертвования</t>
+        </is>
+      </c>
+      <c r="D27" s="6" t="inlineStr">
+        <is>
+          <t>≈ 5 000 ₽/мес</t>
+        </is>
+      </c>
+      <c r="E27" s="7" t="n">
+        <v>5000</v>
+      </c>
+      <c r="F27" s="8" t="inlineStr">
+        <is>
+          <t>Регулярные пожертвования.</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
+          <t>Отношения (быт, совместное время)</t>
+        </is>
+      </c>
+      <c r="B28" s="4">
+        <f>SUM(E28:E29)</f>
+        <v/>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>Выходные: кафе, прогулки, покупки</t>
+        </is>
+      </c>
+      <c r="D28" s="6" t="inlineStr">
+        <is>
+          <t>6 000 ₽ × 4 раза/мес = 24 000 ₽ ⚠</t>
+        </is>
+      </c>
+      <c r="E28" s="7" t="n">
+        <v>24000</v>
+      </c>
+      <c r="F28" s="8" t="inlineStr">
+        <is>
+          <t>Совместные вылазки по выходным + совместный быт дома. Проверь: если быт включает продукты — пересекается с «Питанием».</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="9" t="n"/>
+      <c r="B29" s="9" t="n"/>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>Совместный быт дома</t>
+        </is>
+      </c>
+      <c r="D29" s="6" t="inlineStr">
+        <is>
+          <t>≈ 30 000 ₽/мес ⚠</t>
+        </is>
+      </c>
+      <c r="E29" s="7" t="n">
+        <v>30000</v>
+      </c>
+      <c r="F29" s="9" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
           <t>Поездки</t>
         </is>
       </c>
-      <c r="B28" s="4">
-        <f>SUM(E28:E28)</f>
-        <v/>
-      </c>
-      <c r="C28" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D28" s="5" t="inlineStr">
+      <c r="B30" s="4">
+        <f>SUM(E30:E30)</f>
+        <v/>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>Перелёты / поездки</t>
+        </is>
+      </c>
+      <c r="D30" s="6" t="inlineStr">
         <is>
           <t>⚠ уточни (чем отлич. от «Отдых»?)</t>
         </is>
       </c>
-      <c r="E28" s="6" t="n">
+      <c r="E30" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="F28" s="7" t="inlineStr">
-        <is>
-          <t>Пока не заполнено. Уточни, чем отличается от «Отдыха» — если это перелёты (Азия/домой), посчитаем отдельно.</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="9" t="inlineStr">
+      <c r="F30" s="8" t="inlineStr">
+        <is>
+          <t>Пока не заполнено. Уточни, чем отличается от «Отдыха» (например, перелёты Азия/домой).</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="10" t="inlineStr">
         <is>
           <t>ИТОГО расходов / мес</t>
         </is>
       </c>
-      <c r="B29" s="10">
-        <f>SUM(E3:E28)</f>
-        <v/>
-      </c>
-      <c r="C29" s="11" t="n"/>
-      <c r="D29" s="11" t="n"/>
-      <c r="E29" s="11" t="n"/>
-      <c r="F29" s="11" t="n"/>
-    </row>
-    <row r="31">
-      <c r="A31" s="12" t="inlineStr">
+      <c r="B31" s="11">
+        <f>SUM(E3:E30)</f>
+        <v/>
+      </c>
+      <c r="C31" s="12" t="n"/>
+      <c r="D31" s="12" t="n"/>
+      <c r="E31" s="12" t="n"/>
+      <c r="F31" s="12" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="13" t="inlineStr">
         <is>
           <t>⚠ — оценка/допущение, поправь под себя. Разовые покупки делятся на срок (÷ мес).</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="12" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="13" t="inlineStr">
         <is>
           <t>Не заполнено (нужны твои цифры): Жильё, Бизнес (личный бренд), Поездки.</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="12" t="inlineStr">
-        <is>
-          <t>«Отдых» и «Поездки» пока дублируют смысл — уточни разницу, иначе объединим.</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="12" t="inlineStr">
-        <is>
-          <t>Отношения: 4 вылазки/мес × 6 000 — если вылазок больше/меньше, поправь.</t>
+    <row r="35">
+      <c r="A35" s="13" t="inlineStr">
+        <is>
+          <t>Гаджеты разбиты на устройства; после закупки (3 мес) останется только связь/интернет.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="27">
-    <mergeCell ref="F17:F19"/>
+  <mergeCells count="26">
     <mergeCell ref="A8:A10"/>
-    <mergeCell ref="A17:A19"/>
-    <mergeCell ref="A29"/>
     <mergeCell ref="B11:B12"/>
     <mergeCell ref="A5:A7"/>
-    <mergeCell ref="F20:F21"/>
-    <mergeCell ref="B14:B15"/>
     <mergeCell ref="B5:B7"/>
     <mergeCell ref="F8:F10"/>
+    <mergeCell ref="B14:B17"/>
+    <mergeCell ref="A31"/>
     <mergeCell ref="A33:F33"/>
-    <mergeCell ref="F26:F27"/>
-    <mergeCell ref="A26:A27"/>
-    <mergeCell ref="A32:F32"/>
-    <mergeCell ref="A14:A15"/>
-    <mergeCell ref="A31:F31"/>
-    <mergeCell ref="A20:A21"/>
+    <mergeCell ref="F22:F23"/>
+    <mergeCell ref="A19:A21"/>
+    <mergeCell ref="A35:F35"/>
+    <mergeCell ref="B28:B29"/>
+    <mergeCell ref="F19:F21"/>
+    <mergeCell ref="A22:A23"/>
+    <mergeCell ref="F28:F29"/>
+    <mergeCell ref="A14:A17"/>
+    <mergeCell ref="B8:B10"/>
     <mergeCell ref="A34:F34"/>
-    <mergeCell ref="B8:B10"/>
-    <mergeCell ref="B20:B21"/>
     <mergeCell ref="F5:F7"/>
     <mergeCell ref="F11:F12"/>
-    <mergeCell ref="F14:F15"/>
-    <mergeCell ref="B17:B19"/>
+    <mergeCell ref="F14:F17"/>
+    <mergeCell ref="B22:B23"/>
+    <mergeCell ref="A28:A29"/>
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="B26:B27"/>
+    <mergeCell ref="B19:B21"/>
     <mergeCell ref="A11:A12"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Fill housing (33000), trips (20000), lower visas (12500); total 345166
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WQtgSHTUBUwP9xHzFTYxiY
</commit_message>
<xml_diff>
--- a/decomposition_expenses.xlsx
+++ b/decomposition_expenses.xlsx
@@ -149,7 +149,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -176,6 +176,8 @@
     <xf numFmtId="164" fontId="8" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -608,11 +610,11 @@
       </c>
       <c r="D3" s="6" t="inlineStr">
         <is>
-          <t>⚠ уточни сумму аренды в месяц</t>
+          <t>33 000 ₽/мес</t>
         </is>
       </c>
       <c r="E3" s="7" t="n">
-        <v>0</v>
+        <v>33000</v>
       </c>
       <c r="F3" s="8" t="inlineStr">
         <is>
@@ -679,8 +681,8 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="9" t="n"/>
-      <c r="B6" s="9" t="n"/>
+      <c r="A6" s="14" t="n"/>
+      <c r="B6" s="14" t="n"/>
       <c r="C6" s="5" t="inlineStr">
         <is>
           <t>Танцы: рейвы, джемы, съёмки клипа</t>
@@ -694,11 +696,11 @@
       <c r="E6" s="7" t="n">
         <v>2000</v>
       </c>
-      <c r="F6" s="9" t="n"/>
+      <c r="F6" s="14" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="9" t="n"/>
-      <c r="B7" s="9" t="n"/>
+      <c r="A7" s="15" t="n"/>
+      <c r="B7" s="15" t="n"/>
       <c r="C7" s="5" t="inlineStr">
         <is>
           <t>Обучение (гипноз, ретриты)</t>
@@ -712,7 +714,7 @@
       <c r="E7" s="7" t="n">
         <v>33333</v>
       </c>
-      <c r="F7" s="9" t="n"/>
+      <c r="F7" s="15" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
@@ -744,8 +746,8 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="9" t="n"/>
-      <c r="B9" s="9" t="n"/>
+      <c r="A9" s="14" t="n"/>
+      <c r="B9" s="14" t="n"/>
       <c r="C9" s="5" t="inlineStr">
         <is>
           <t>Бады</t>
@@ -759,11 +761,11 @@
       <c r="E9" s="7" t="n">
         <v>5000</v>
       </c>
-      <c r="F9" s="9" t="n"/>
+      <c r="F9" s="14" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="9" t="n"/>
-      <c r="B10" s="9" t="n"/>
+      <c r="A10" s="15" t="n"/>
+      <c r="B10" s="15" t="n"/>
       <c r="C10" s="5" t="inlineStr">
         <is>
           <t>Мухоморы, микродозинг и прочее</t>
@@ -777,7 +779,7 @@
       <c r="E10" s="7" t="n">
         <v>3000</v>
       </c>
-      <c r="F10" s="9" t="n"/>
+      <c r="F10" s="15" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
@@ -809,8 +811,8 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="9" t="n"/>
-      <c r="B12" s="9" t="n"/>
+      <c r="A12" s="15" t="n"/>
+      <c r="B12" s="15" t="n"/>
       <c r="C12" s="5" t="inlineStr">
         <is>
           <t>Такси Nusa Dua ↔ Nuanu</t>
@@ -824,7 +826,7 @@
       <c r="E12" s="7" t="n">
         <v>15000</v>
       </c>
-      <c r="F12" s="9" t="n"/>
+      <c r="F12" s="15" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
@@ -885,8 +887,8 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="9" t="n"/>
-      <c r="B15" s="9" t="n"/>
+      <c r="A15" s="14" t="n"/>
+      <c r="B15" s="14" t="n"/>
       <c r="C15" s="5" t="inlineStr">
         <is>
           <t>Колонки</t>
@@ -900,11 +902,11 @@
       <c r="E15" s="7" t="n">
         <v>1667</v>
       </c>
-      <c r="F15" s="9" t="n"/>
+      <c r="F15" s="14" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="9" t="n"/>
-      <c r="B16" s="9" t="n"/>
+      <c r="A16" s="14" t="n"/>
+      <c r="B16" s="14" t="n"/>
       <c r="C16" s="5" t="inlineStr">
         <is>
           <t>Оперативка 16 ГБ</t>
@@ -918,11 +920,11 @@
       <c r="E16" s="7" t="n">
         <v>1666</v>
       </c>
-      <c r="F16" s="9" t="n"/>
+      <c r="F16" s="14" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="9" t="n"/>
-      <c r="B17" s="9" t="n"/>
+      <c r="A17" s="15" t="n"/>
+      <c r="B17" s="15" t="n"/>
       <c r="C17" s="5" t="inlineStr">
         <is>
           <t>Оператор связи + домашний интернет</t>
@@ -936,7 +938,7 @@
       <c r="E17" s="7" t="n">
         <v>2000</v>
       </c>
-      <c r="F17" s="9" t="n"/>
+      <c r="F17" s="15" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
@@ -997,8 +999,8 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="9" t="n"/>
-      <c r="B20" s="9" t="n"/>
+      <c r="A20" s="14" t="n"/>
+      <c r="B20" s="14" t="n"/>
       <c r="C20" s="5" t="inlineStr">
         <is>
           <t>Продукты</t>
@@ -1012,11 +1014,11 @@
       <c r="E20" s="7" t="n">
         <v>12000</v>
       </c>
-      <c r="F20" s="9" t="n"/>
+      <c r="F20" s="14" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="9" t="n"/>
-      <c r="B21" s="9" t="n"/>
+      <c r="A21" s="15" t="n"/>
+      <c r="B21" s="15" t="n"/>
       <c r="C21" s="5" t="inlineStr">
         <is>
           <t>Доставка</t>
@@ -1030,7 +1032,7 @@
       <c r="E21" s="7" t="n">
         <v>2000</v>
       </c>
-      <c r="F21" s="9" t="n"/>
+      <c r="F21" s="15" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
@@ -1062,8 +1064,8 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="9" t="n"/>
-      <c r="B23" s="9" t="n"/>
+      <c r="A23" s="15" t="n"/>
+      <c r="B23" s="15" t="n"/>
       <c r="C23" s="5" t="inlineStr">
         <is>
           <t>Девушке</t>
@@ -1077,7 +1079,7 @@
       <c r="E23" s="7" t="n">
         <v>5000</v>
       </c>
-      <c r="F23" s="9" t="n"/>
+      <c r="F23" s="15" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
@@ -1154,11 +1156,11 @@
       </c>
       <c r="D26" s="6" t="inlineStr">
         <is>
-          <t>≈ 20 000 ₽/мес ⚠ (перенос, подтверди)</t>
+          <t>≈ 12 500 ₽/мес</t>
         </is>
       </c>
       <c r="E26" s="7" t="n">
-        <v>20000</v>
+        <v>12500</v>
       </c>
       <c r="F26" s="8" t="inlineStr">
         <is>
@@ -1225,8 +1227,8 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="9" t="n"/>
-      <c r="B29" s="9" t="n"/>
+      <c r="A29" s="15" t="n"/>
+      <c r="B29" s="15" t="n"/>
       <c r="C29" s="5" t="inlineStr">
         <is>
           <t>Совместный быт дома</t>
@@ -1240,7 +1242,7 @@
       <c r="E29" s="7" t="n">
         <v>30000</v>
       </c>
-      <c r="F29" s="9" t="n"/>
+      <c r="F29" s="15" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
@@ -1259,11 +1261,11 @@
       </c>
       <c r="D30" s="6" t="inlineStr">
         <is>
-          <t>⚠ уточни (чем отлич. от «Отдых»?)</t>
+          <t>≈ 20 000 ₽/мес</t>
         </is>
       </c>
       <c r="E30" s="7" t="n">
-        <v>0</v>
+        <v>20000</v>
       </c>
       <c r="F30" s="8" t="inlineStr">
         <is>
@@ -1286,6 +1288,7 @@
       <c r="E31" s="12" t="n"/>
       <c r="F31" s="12" t="n"/>
     </row>
+    <row r="32"/>
     <row r="33">
       <c r="A33" s="13" t="inlineStr">
         <is>
@@ -1313,10 +1316,10 @@
     <mergeCell ref="B11:B12"/>
     <mergeCell ref="A5:A7"/>
     <mergeCell ref="B5:B7"/>
+    <mergeCell ref="A31"/>
+    <mergeCell ref="B14:B17"/>
+    <mergeCell ref="A33:F33"/>
     <mergeCell ref="F8:F10"/>
-    <mergeCell ref="B14:B17"/>
-    <mergeCell ref="A31"/>
-    <mergeCell ref="A33:F33"/>
     <mergeCell ref="F22:F23"/>
     <mergeCell ref="A19:A21"/>
     <mergeCell ref="A35:F35"/>

</xml_diff>